<commit_message>
Fix VCP and Make field locators with alternative selector fallback
- VCP field now found using input[id*='VCP'] pattern as primary fallback
- Added robust error handling to try multiple selector patterns
- Both VCP and Make fields now use waitFor with visible state
- Tests 50-53 all pass successfully with all form fields filled
</commit_message>
<xml_diff>
--- a/testData/Buyer_PO_Upload/PO Summary format1.xlsx
+++ b/testData/Buyer_PO_Upload/PO Summary format1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://perfectbss-my.sharepoint.com/personal/thilina_perfectbss_com/Documents/Desktop/Apperal_Module/testData/Buyer_PO_Upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{40B3E097-4904-4243-8D7D-6D3250CCD28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{581A16CB-31E7-4E4A-AB68-7223008A41E7}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{40B3E097-4904-4243-8D7D-6D3250CCD28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4ADD2A5-25E7-4B93-AA88-0ECB55ADEBC9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="54">
   <si>
     <t xml:space="preserve">Buyer </t>
   </si>
@@ -106,9 +106,6 @@
     <t>Season</t>
   </si>
   <si>
-    <t>SS25 PH02</t>
-  </si>
-  <si>
     <t>UK</t>
   </si>
   <si>
@@ -184,16 +181,22 @@
     <t>L</t>
   </si>
   <si>
-    <t>QA0001</t>
-  </si>
-  <si>
-    <t>QA 2</t>
-  </si>
-  <si>
-    <t>QA2</t>
-  </si>
-  <si>
-    <t>QA2-T001</t>
+    <t>Buyer 001</t>
+  </si>
+  <si>
+    <t>BUY0001</t>
+  </si>
+  <si>
+    <t>BUY2</t>
+  </si>
+  <si>
+    <t>BUY_C2</t>
+  </si>
+  <si>
+    <t>BUY25 SE02</t>
+  </si>
+  <si>
+    <t>PONO</t>
   </si>
 </sst>
 </file>
@@ -678,7 +681,7 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -700,7 +703,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -722,7 +725,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -810,13 +813,13 @@
         <v>7</v>
       </c>
       <c r="D10" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="F10" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="G10" s="19"/>
       <c r="H10" s="19"/>
@@ -833,10 +836,10 @@
     </row>
     <row r="11" spans="1:18" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>11</v>
@@ -1265,7 +1268,7 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -1276,7 +1279,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -1287,7 +1290,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1298,7 +1301,7 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1309,7 +1312,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -1388,10 +1391,10 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>11</v>
@@ -1590,31 +1593,31 @@
         <v>7</v>
       </c>
       <c r="D16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="I16" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="J16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
@@ -1625,10 +1628,10 @@
     </row>
     <row r="17" spans="1:18" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>11</v>
@@ -1774,10 +1777,10 @@
     </row>
     <row r="20" spans="1:18" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>32</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>33</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>11</v>
@@ -1923,10 +1926,10 @@
     </row>
     <row r="23" spans="1:18" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>34</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>35</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>11</v>
@@ -2072,10 +2075,10 @@
     </row>
     <row r="26" spans="1:18" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>11</v>

</xml_diff>